<commit_message>
feat(resources): import reviewed health support resources
</commit_message>
<xml_diff>
--- a/docs/resource_total.xlsx
+++ b/docs/resource_total.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S65"/>
+  <dimension ref="A1:S88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -434,7 +434,7 @@
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="46" customWidth="1" min="13" max="13"/>
     <col width="6" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
     <col width="6" customWidth="1" min="16" max="16"/>
     <col width="8" customWidth="1" min="17" max="17"/>
     <col width="6" customWidth="1" min="18" max="18"/>
@@ -6746,6 +6746,2237 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>高齡孕婦掌握7原則 助安心懷孕平安生產</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/Pages/Detail.aspx?nodeid=4306&amp;pid=14146</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>國民健康署整理高齡孕婦在產檢、營養、體重、慢性病控制與生活管理上的重要原則，協助降低妊娠相關風險。</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>官方衛教文章</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>孕期</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>孕產與嬰幼兒照護</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>高齡孕婦, 高齡妊娠, 產前檢查, 妊娠風險, 孕期保健</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>高：中央衛生主管機關官方衛教。</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>屬一般衛教；個人風險與檢查安排仍應由婦產科醫師評估。</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>產前遺傳診斷</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/Pages/List.aspx?nodeid=197</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>說明產前遺傳診斷的補助對象、檢查項目與減免額度；34歲以上孕婦及其他高風險族群可依條件申請。</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>官方服務資訊</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>孕期</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>孕產與嬰幼兒照護</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>產前遺傳診斷, 羊膜穿刺, 染色體, 遺傳疾病, 高齡孕婦, 補助</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>高：中央衛生主管機關官方補助與服務資訊。</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>補助資格與金額可能調整，應以頁面最新公告為準。</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>補助</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>孕婦健康手冊</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/Pages/EBook.aspx?nodeid=1142</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>國民健康署官方孕婦健康手冊，配合產檢時程提供健康紀錄、孕期保健、檢查與警訊等完整資訊。</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>官方手冊</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>孕期</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>孕產與嬰幼兒照護</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>孕婦健康手冊, 產檢, 孕期保健, 高危險妊娠, 孕婦</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>高：官方孕產婦基礎指引，可作高齡妊娠的核心總覽資源。</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>內容涵蓋所有孕婦，不只高齡孕婦；育伴可在高齡妊娠主題中作基礎入口。</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>認識高危險妊娠</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://www.ntuh.gov.tw/obgy/Faq.action?agroup=a&amp;fid=63&amp;q_type=A05</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>臺大醫院婦產部說明高危險妊娠定義與常見危險因子，包括孕婦年齡、體重、既有疾病與妊娠併發症。</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>醫療衛教</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>醫療院所</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>國立臺灣大學醫學院附設醫院 婦產部</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>孕期</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>孕產與嬰幼兒照護</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>高危險妊娠, 高齡孕婦, 妊娠高血壓, 妊娠糖尿病, 產科</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>高：醫學中心婦產科專業衛教。</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>高齡只是高危險妊娠的其中一項因子，實際風險需依個人病史與孕況評估。</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>羊膜穿刺術之照護</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://ihealth.vghtpe.gov.tw/media/637</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>臺北榮總說明羊膜穿刺目的、適用情況、檢查流程與檢查後照護，並列出需立即就醫的警訊。</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>醫療衛教</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>醫療院所</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>臺北榮民總醫院</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>孕期</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>孕產與嬰幼兒照護</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>羊膜穿刺, 產前診斷, 染色體異常, 高齡孕婦, 檢查照護</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>高：醫學中心醫療衛教，適合作為檢查前後照護參考。</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>是否接受羊膜穿刺應與產科醫師或遺傳諮詢專業人員討論。</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>NIPT可以取代羊膜穿刺作為確診方法嗎？</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/Pages/Detail.aspx?nodeid=127&amp;pid=7795</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>國民健康署說明非侵入性胎兒染色體檢查（NIPT）屬篩檢而非確診，不能直接取代羊膜穿刺或絨毛膜採樣。</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>官方QA</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>孕期</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>孕產與嬰幼兒照護</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>NIPT, 羊膜穿刺, 染色體篩檢, 產前檢查, 高齡孕婦</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>高：官方風險溝通與檢查定位說明。</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>檢測技術持續演進；個別檢測選擇仍應依醫師與遺傳諮詢建議。</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>試管嬰兒專區</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/Pages/List.aspx?nodeid=314</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>國民健康署人工生殖官方入口，整合試管嬰兒補助、QA、人工生殖機構名單、申辦說明等資訊。</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>官方專區</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>備孕／不孕療程</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>備孕與生殖</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>人工生殖, 試管嬰兒, IVF, 不孕症, 補助, 人工生殖機構</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>高：人工生殖政策與補助的官方主要入口。</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>專區以試管嬰兒為主；人工授精（IUI）療程資訊可搭配醫療院所資源。</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>不孕症試管嬰兒補助3.0方案</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/Pages/Detail.aspx?nodeid=500&amp;pid=14149</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>國民健康署最新試管嬰兒補助方案，說明資格、補助額度、申請次數與療程規範。</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>官方補助資訊</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>備孕／不孕療程</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>備孕與生殖</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>試管嬰兒補助, IVF, 不孕症, 人工生殖, 補助3.0</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>高：官方補助規範，2026年仍持續更新。</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>政策與補助額度可能修正，正式申請前需確認最新版本。</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>補助</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>不孕症試管嬰兒補助3.0方案QA問答集</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/EngPages/Detail.aspx?nodeid=500&amp;pid=15871</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>以問答方式整理試管嬰兒補助資格、療程、申請與常見特殊情況，適合民眾快速確認細節。</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>官方QA</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>備孕／不孕療程</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>備孕與生殖</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>IVF補助, 試管嬰兒, 不孕症, QA, 補助資格</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>高：官方QA文件，適合搭配補助方案主頁使用。</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>目前搜尋結果導向國健署英文頁面但內容與附件為官方資料；如取得中文直連可再替換。</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>特約人工生殖機構及許可人工生殖機構名單</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/Pages/Detail.aspx?nodeid=500&amp;pid=14267</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>提供試管嬰兒補助特約人工生殖機構及衛福部許可人工生殖機構最新名單，方便查找合法院所。</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>官方名單</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>備孕／不孕療程</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>備孕與生殖</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>人工生殖機構, 試管嬰兒, IVF, 合法院所, 特約機構</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>高：主管機關官方許可與特約機構名單。</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>院所名單會更新；網站應以最新更新日期為準。</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>人工授精</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://www.ntuh.gov.tw/obgy/Fpage.action?fid=8625&amp;muid=7913</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>臺大醫院婦產部說明人工授精（IUI）的原理、療程流程、適用條件、費用範圍與一般成功率。</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>醫療衛教</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>醫療院所</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>國立臺灣大學醫學院附設醫院 婦產部</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>備孕／不孕療程</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>備孕與生殖</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>人工授精, IUI, 排卵, 不孕症, 療程流程, 生殖醫學</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>高：醫學中心生殖醫學專業資訊，直接涵蓋人工授精。</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>成功率與費用依年齡、診斷、用藥與院所而異，應以個別醫療評估為準。</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>台灣生殖醫學會</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://www.tsrm.org.tw/</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>台灣生殖醫學專業學會入口，提供人工生殖、生殖醫學專業資訊、政策訊息與相關衛教資源。</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>專業學會入口</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>專業學會</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>台灣生殖醫學會</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>備孕／不孕療程</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>備孕與生殖</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>生殖醫學, 不孕症, 人工生殖, IVF, IUI, 專業學會</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>高：台灣生殖醫學專業學會。</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>首頁偏專業與學術資訊；育伴可後續再細拆適合一般民眾閱讀的衛教文章。</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>顱顏百科－唇腭裂</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://www.nncf.org/family/clp/clp_intro</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>羅慧夫顱顏基金會的唇顎裂總覽，涵蓋疾病介紹、療程費用與資源、治療照顧與常見問題。</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>疾病專題入口</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>專業基金會</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>財團法人羅慧夫顱顏基金會</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>新生兒至青少年</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>兒科疾病與照護</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>唇顎裂, 唇裂, 顎裂, 顱顏, 治療, 照護</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>高：台灣長期專注顱顏患者醫療與支持服務之基金會。</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>適合作為唇顎裂主題總入口；個別治療仍需依顱顏醫療團隊評估。</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>唇腭裂哺餵技巧</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://www.nncf.org/family/clp/clp_treatment/Introduction_feedskill</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>說明唇顎裂寶寶的母乳、奶瓶、奶嘴選擇、餵食姿勢、拍嗝與口腔清潔等實作技巧。</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>照護指南</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>專業基金會</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>財團法人羅慧夫顱顏基金會</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>新生兒／嬰兒</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>兒科疾病與照護</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>唇顎裂餵食, 特殊奶瓶, 哺乳, 奶嘴, 吞嚥, 新生兒照護</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>高：針對唇顎裂家庭的專門照護資源，實作性高。</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>若嬰兒出現吞嚥、呼吸、體重增加等問題，應尋求顱顏團隊、兒科或語言治療師評估。</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>學齡前</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>唇腭裂術前準備及術後照顧</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://www.nncf.org/family/clp/clp_treatment/Introduction_surgery_prepare</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>整理唇裂、顎裂及相關顱顏手術的術前準備、傷口清潔、餵食、姿勢與術後照護重點。</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>照護指南</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>專業基金會</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>財團法人羅慧夫顱顏基金會</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>嬰幼兒至青少年</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>兒科疾病與照護</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>唇顎裂手術, 術前準備, 術後照護, 傷口照護, 餵食</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>高：唇顎裂手術照護專門資源。</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>不同手術方式與院所指示可能不同，術後照護應以主治團隊指示優先。</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>唇腭裂療程費用及社會資源</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>https://www.nncf.org/family/clp/clp_intro/Introduction_cost_society</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>整理唇顎裂療程費用、重大傷病、身心障礙資格與基金會交通及醫療補助等社會資源。</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>補助／社會資源</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>專業基金會</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>財團法人羅慧夫顱顏基金會</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>新生兒至成人</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>兒科疾病與照護</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>唇顎裂補助, 重大傷病, 身心障礙, 醫療費用, 交通補助</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>高：專門服務顱顏家庭的社福與醫療支持資訊。</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>補助資格與福利依個案、縣市及當期規定而異，申請前應再向主管機關確認。</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>補助</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>顱顏照護指南－醫師及專家文章整理</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>https://www.nncf.org/news/index/1/tx7yl</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>彙整顱顏醫療專家文章，涵蓋唇顎裂餵食、口腔、中耳炎、語言治療、心理與整體醫療等議題。</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>專家文章入口</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>醫療專業／基金會</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>財團法人羅慧夫顱顏基金會</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>嬰幼兒至青少年</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>兒科疾病與照護</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>唇顎裂, 語言治療, 口腔照護, 中耳炎, 心理支持, 顱顏醫療</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>高：文章作者多為長庚顱顏相關醫師、治療師與專業人員。</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>屬集合頁；育伴後續可再拆出最具家長行動價值的單篇文章。</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>長庚顱顏中心</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>https://www.cgmh.org.tw/tw/Systems/BranchInfo/3/32000/32500/32540</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>長庚顱顏中心提供唇顎裂及各類顱顏畸形的跨專科整合醫療，包含顱顏外科、齒顎矯正與語言治療等。</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>醫療服務入口</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>醫療院所</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>長庚醫療財團法人 顱顏中心</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>新生兒至成人</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>兒科疾病與照護</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>唇顎裂, 顱顏中心, 整合醫療, 顱顏外科, 齒顎矯正, 語言治療</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>高：大型醫學中心專門顱顏整合團隊。</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>屬就醫入口，實際療程與時程需經團隊評估。</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>全齡</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>桃園／全台可就醫</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>兒童發展篩檢服務</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/Pages/List.aspx?nodeid=4816</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>國民健康署兒童發展篩檢官方專區，整合篩檢服務、量表、懶人包、轉介流程與相關說明。</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>官方專區</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>嬰幼兒／學齡前</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>發展與早療</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>兒童發展篩檢, 發展遲緩, 早療, 聯合評估, 發展里程碑</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>高：現行兒童發展篩檢政策的官方核心入口。</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>篩檢結果不是診斷；疑似異常需依流程轉介聯合評估。</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>學齡前</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>兒童發展篩檢量表</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/Pages/List.aspx?nodeid=4821</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>提供不同年齡層的標準化兒童發展篩檢量表與工具，涵蓋6個月至7歲等多個階段。</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>官方量表</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>嬰幼兒／學齡前</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>發展與早療</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>發展篩檢量表, 兒童發展, 發展里程碑, 早期發現, 0-7歲</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>高：國民健康署與馬偕紀念醫院合作建置之本土化標準化工具。</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>正式兒童發展篩檢應由具資格醫師執行；家長可作理解與準備用途。</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>學齡前</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>兒童發展聯合評估中心名單</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>https://www.hpa.gov.tw/1602/548/n</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>提供全台兒童發展聯合評估中心最新名單，供疑似發展遲緩兒童接受跨專科評估與診斷。</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>官方名單</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>衛生福利部國民健康署</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>嬰幼兒／學齡前</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>發展與早療</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>聯合評估中心, 發展遲緩, 兒童發展, 早療, 評估</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>高：主管機關官方中心名單，2026年持續更新。</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>中心名單與服務量能可能更新；預約前應確認各院所門診資訊。</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>學齡前</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>孩子是否發展遲緩？認識發展遲緩及早期療育補助</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>https://www.gov.tw/News_Content_26_578611</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>我的E政府以家長流程角度整理發展遲緩辨識、診斷、通報、療育與交通／療育費用補助申請。</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>官方懶人包</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>我的E政府</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>嬰幼兒／學齡前</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>發展與早療</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>早療補助, 發展遲緩, 交通費, 療育費, 申請流程, 通報</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>高：政府整合式申辦說明，家長行動導向清楚。</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>補助金額與申請單位依縣市不同，應以所在地政府最新規定為準。</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>學齡前</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>補助</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>臺北榮總兒童發展評估中心－早期療育資源介紹</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>https://wd.vghtpe.gov.tw/PMREIP/Fpage.action?fid=9954&amp;muid=10308</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>介紹早療的醫療復健、日間療育、社福與家庭支持等服務型態，幫助家長理解完成評估後有哪些資源可使用。</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>醫療衛教</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>醫療院所</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>臺北榮民總醫院 兒童發展評估中心</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>嬰幼兒／學齡前</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>發展與早療</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>早期療育, 發展遲緩, 復健, 日間療育, 家庭支持, 兒童發展</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>高：醫學中心兒童發展評估專業團隊。</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>北部院所內容可作全台概念參考；實際療育據點仍應依所在地資源選擇。</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>學齡前</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>北部／全台參考</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(resources): import reviewed ADHD resources
</commit_message>
<xml_diff>
--- a/docs/resource_total.xlsx
+++ b/docs/resource_total.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S88"/>
+  <dimension ref="A1:S102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -428,15 +428,15 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="46" customWidth="1" min="13" max="13"/>
-    <col width="6" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
     <col width="6" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
     <col width="6" customWidth="1" min="18" max="18"/>
     <col width="6" customWidth="1" min="19" max="19"/>
   </cols>
@@ -8977,6 +8977,1364 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ADHD注意力不足過動症相關衛教資源</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>https://www.mohw.gov.tw/cp-189-212-1.html</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>衛生福利部心理健康資源頁，將 ADHD 衛教列為心理健康促進資源之一，提供疾病認識、早期治療與支持照顧者的官方入口。</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>官方資源入口</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>政府／官方</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>衛生福利部</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>兒童至成人</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>ADHD, 注意力不足, 過動, 心理健康, 早期治療, 照顧者支持</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>高：中央衛生主管機關心理健康司官方入口。</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>此頁為心理健康綜合入口，ADHD 為其中一項；育伴可再搭配更細的專業衛教與就醫資源。</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>學齡前, 國小, 國中, 高中, 成人</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>家長, 兒童</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ADHD注意力不足過動症衛教專欄</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>https://www.tscap.org.tw/TW/NewsColumn/ugC_News.asp?hidNewsCatID=6</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>台灣兒童青少年精神醫學會 ADHD 專區，彙整症狀、診斷、治療、藥物、親職、校園支持與迷思澄清等內容。</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>專業專區</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>專業學會</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>台灣兒童青少年精神醫學會</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>兒童／青少年</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>ADHD, 診斷, 治療, 藥物, 親職, 校園支持, 迷思</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>高：台灣兒童青少年精神醫學專業學會官方衛教專區。</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>專區內同主題文章較多，育伴應精選不同用途的代表資源，不需全量收錄。</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>國小, 國中, 高中</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>家長, 教師, 兒童</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>注意力不足過動症：診斷標準、病因與盛行率</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>https://www.tscap.org.tw/TW/NewsColumn/ugC_News_Detail.asp?hidNewsCatID=6&amp;hidNewsID=205</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>由國家衛生研究院論壇撰文、台灣兒童青少年精神醫學會審評，介紹 ADHD 的核心症狀、病因、盛行率與何時應尋求專業評估。</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>專業衛教文章</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>專業學會／研究機構</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>台灣兒童青少年精神醫學會</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>兒童／青少年</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>ADHD症狀, 診斷, 病因, 盛行率, 注意力不集中, 過動, 衝動</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>高：由專業學會審評，適合建立疾病基本認識。</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>文章內部分段仍引用較舊診斷版本文字；正式診斷應以現行專業評估與最新診斷準則為準。</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>國小, 國中, 高中</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>家長, 教師, 兒童</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>注意力不足過動症需要治療嗎？接下來該怎麼辦、怎麼治療</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>https://www.tscap.org.tw/TW/NewsColumn/ugC_News_Detail.asp?hidNewsCatID=6&amp;hidNewsID=206</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>說明 ADHD 的評估流程與整合性治療，包含藥物、行為治療、學校環境支持，以及不同年齡層的治療考量。</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>專業衛教文章</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>專業學會／研究機構</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>台灣兒童青少年精神醫學會</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>兒童／青少年</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>ADHD治療, 藥物治療, 行為治療, 學校支持, 兒童心智科</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>高：由台灣兒童青少年精神醫學會審評，聚焦治療決策。</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>治療方式需依年齡、功能受損程度、共病與家庭需求，由兒童青少年精神專科醫師共同規劃。</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>國小, 國中, 高中</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>家長, 兒童</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>全台兒童青少年精神專科醫師分佈</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>https://www.tscap.org.tw/TW/Retail/ugC_Retail.asp</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>可依地區與縣市查找兒童青少年精神專科醫師，適合疑似 ADHD、需要診斷評估或持續治療的家庭尋找專科資源。</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>專科醫師查詢</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>專業學會</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>台灣兒童青少年精神醫學會</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>兒童／青少年</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>兒童心智科, 兒童青少年精神科, ADHD評估, 醫師查詢, 就醫</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>高：兒童青少年精神專業學會提供的專科醫師分佈資料。</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>實際門診時段與是否收治 ADHD 應再向醫療院所確認。</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>學齡前, 國小, 國中, 高中</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>家長, 兒童</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ADHD注意力不足過動症資料網推薦</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>https://www.health.taichung.gov.tw/2349646/post</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>臺中市政府衛生局 ADHD 專區推薦台灣兒童青少年精神醫學會所屬資料網，內容涵蓋常見迷思、教養、治療、藥物與醫療資源。</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>政府資源導覽</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>地方政府／官方</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>臺中市政府衛生局</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>兒童／青少年</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>ADHD資料網, 迷思, 教養, 治療, 藥物, 醫療資源</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>高：地方衛生主管機關於 2026 年更新的 ADHD 導覽資源。</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>屬推薦／導覽頁，核心醫療資訊仍應以專業學會與醫療院所原始內容為準。</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>國小, 國中, 高中</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>家長, 教師</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>領有 ADHD 診斷證明，可以申請特教服務或教育補助嗎？</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>https://www.tyc.edu.tw/News_Content.aspx?n=5180&amp;s=1468476</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>桃園市教育局說明 ADHD 醫療診斷與學校特殊教育鑑定的差異，以及需要特教服務時應向學校輔導室提出情緒行為障礙鑑定安置申請。</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>教育權益說明</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>地方政府／教育</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>桃園市政府教育局</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>學齡兒童／青少年</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>ADHD, 特教服務, 情緒行為障礙, 鑑輔會, 教育補助, 學校輔導</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>高：教育主管機關於 2026 年更新，直接回答家長常見教育權益問題。</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>各縣市鑑定流程與補助細節可能不同；非桃園家庭應再確認所在地教育局規定。</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>國小, 國中, 高中</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>桃園市／全台參考</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>政策</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>家長, 教師</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>注意力缺陷過動症20問與 ADHD 青少年教材</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>https://web.terc.tp.edu.tw/</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>臺北市東區特教資源中心提供「注意力缺陷過動症20問」及適用國高中的 ADHD 青少年組教材，協助教師理解與支持學生。</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>特教教材入口</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>教育專業／地方教育</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>臺北市東區特教資源中心</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>學齡兒童／青少年</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>ADHD教師手冊, 特教, 校園支持, 青少年教材, 注意力缺陷過動症20問</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>高：臺北市教育體系特教資源中心出版／彙整之教材。</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>首頁需進入「教材與出版品」尋找 ADHD 相關教材；不同教材適用年齡不同。</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>國小, 國中, 高中</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>臺北市／全台參考</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>教師, 家長, 兒童</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>注意力缺陷與過動症：大專校園支持方式</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>https://dss.ntu.edu.tw/AboutDisability/D-7</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>臺灣大學資源教室說明 ADHD 對大學生學習與生活的影響，並提供同儕與教學支持策略，例如簡潔指示、具體提醒與學習協助。</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>校園支持指南</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>大學／教育支持</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>國立臺灣大學學生心理輔導中心資源教室</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>大專／成人</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>成人ADHD, 大學生, 校園支持, 學習調整, 注意力, 資源教室</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>高：國立大學身心障礙學生資源教室官方教育支持內容。</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>主要為大專校園情境，不是診斷或治療指引。</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>成人</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>成人, 教師</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>注意力不足過動症｜早期療育中心衛教</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>https://www.hch.gov.tw/?aid=626&amp;iid=1445&amp;page_name=detail&amp;pid=94</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>新竹臺大分院早期療育中心提供 ADHD 衛教資料，由臨床心理專業人員整理，供家長理解注意力與過動相關問題。</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>醫療衛教</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>醫療院所</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>新竹臺大分院早期療育中心</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>幼兒／學齡兒童</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>ADHD, 早療, 臨床心理, 注意力不集中, 過動, 親職</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>高：醫學中心體系早療中心，由臨床心理專業人員提供衛教。</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>衛教資料不能取代完整臨床診斷；幼兒期注意力與活動量需配合發展年齡評估。</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>學齡前, 國小</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>注意力欠缺過動症｜衛教單張</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>https://www.cmuh.cmu.edu.tw/HealthEdus/Detail?no=5623</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>中國醫藥大學附設醫院整理 ADHD 的症狀、常見功能困難與療育方式，並說明藥物及行為治療會依個別困擾程度安排。</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>醫療衛教</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>醫療院所</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>中國醫藥大學附設醫院</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>兒童／青少年</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>ADHD症狀, 行為治療, 藥物治療, 學習, 人際, 情緒</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>高：醫學中心衛教內容，2026 年更新。</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>診斷需排除其他造成注意力或行為問題的原因；治療需個別化。</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>國小, 國中, 高中</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>家長, 兒童</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>ADHD家長手冊</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>https://www.vghtc.gov.tw/UnitPage/RowViewDetail?CompanyID=e8e0488e-54a0-44bf-b10c-d029c423f6e7&amp;UnitDefaultTemplate=1&amp;UnitID=1f26aa21-7dcc-445a-8fd1-c7aba97c3f30&amp;WebRowsID=64227905-a044-415f-a3d1-257b84969812</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>臺中榮總提供 ADHD 家長手冊，包含與醫師溝通、建立結構化日常生活、尋找支持與理解孩子等照護建議。</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>家長手冊</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>醫療院所</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>臺中榮民總醫院</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>兒童／青少年</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>ADHD家長手冊, 親職, 日常結構, 醫病溝通, 家庭支持</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>高：醫學中心提供之家長照護手冊，2025 年更新。</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>頁面可能因網站改版導向院方首頁；若育伴匯入後連結失效，應列入定期連結檢查。</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>國小, 國中, 高中</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>學習教材</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>注意力不集中／ADHD 衛教資源</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>https://webdept.fjuh.fju.edu.tw/FjuhDep/childdev/category/headinfo/adhd/</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>輔大醫院兒童發展評估暨療育中心彙整 ADHD 與注意力不集中相關衛教，包括兒童 ADHD 上下篇、家長篇、居家活動建議與注意力分類。</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>醫療專題入口</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>醫療院所／兒童發展中心</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>輔仁大學附設醫院兒童發展評估暨療育中心</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>幼兒／學齡兒童</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>ADHD, 注意力不集中, 家長篇, 居家活動, 兒童發展, 早療</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>高：兒童發展評估暨療育中心專題頁，2025–2026 年持續更新。</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>專區文章用途不同，育伴未來可再精選「家長篇」與「居家活動」作子資源。</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>學齡前, 國小</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>全台</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>家長</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>臺大醫院兒童心智科／兒童心理衛生服務</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>https://www.ntuh.gov.tw/ccnb/Fpage.action?fid=1651</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>臺大醫院兒童心理衛生中心提供 ADHD 等兒童青少年情緒行為問題的診斷、藥物、心理治療、家長團體、功能評估與社會資源轉介。</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>醫療服務入口</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>醫療院所</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>國立臺灣大學醫學院附設醫院</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>兒童／青少年</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>注意力與過動（ADHD）</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>兒童心智科, ADHD就醫, 心理衡鑑, 行為治療, 家長團體, 藥物治療</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>人工核實</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>高：醫學中心兒童青少年精神醫療專業團隊。</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>屬實際醫療服務入口；門診與團體開設狀況需依院方當期公告。</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>學齡前, 國小, 國中, 高中</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>臺北市／全台可就醫</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>機構</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>家長, 兒童</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>台灣</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>繁體中文</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>